<commit_message>
add cost scenario to example data. drop missing rows from add_object_object_object().
</commit_message>
<xml_diff>
--- a/example_data/connections/connections-input.xlsx
+++ b/example_data/connections/connections-input.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
   <si>
     <t xml:space="preserve">node1</t>
   </si>
@@ -477,7 +477,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.45"/>
@@ -587,6 +587,26 @@
       </c>
       <c r="L3" s="3" t="n">
         <v>1000</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>